<commit_message>
correctly reset guests on import, add example guest file, sort guests on import
</commit_message>
<xml_diff>
--- a/data/example_file.xlsx
+++ b/data/example_file.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ubric\Documents\GitHub\Abiball-Tischordnung\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A956883A-B65F-4B6A-8879-D9B09A0A3C52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C81D96D-69F3-4552-8A2D-BEF438A2D799}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{879EE254-DC9E-4C79-83D5-9A5CB8BE5CFF}"/>
+    <workbookView xWindow="28680" yWindow="4350" windowWidth="29040" windowHeight="15720" xr2:uid="{879EE254-DC9E-4C79-83D5-9A5CB8BE5CFF}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
when importing guests, they are now merged with the existing guests
</commit_message>
<xml_diff>
--- a/data/example_file.xlsx
+++ b/data/example_file.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ubric\Documents\GitHub\Abiball-Tischordnung\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C81D96D-69F3-4552-8A2D-BEF438A2D799}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB7DCDE1-1F89-4E4A-B2D6-F6AB142372EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="4350" windowWidth="29040" windowHeight="15720" xr2:uid="{879EE254-DC9E-4C79-83D5-9A5CB8BE5CFF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{879EE254-DC9E-4C79-83D5-9A5CB8BE5CFF}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -39,28 +39,28 @@
     <t>WunschNachbar2</t>
   </si>
   <si>
-    <t>Erika Mustermann</t>
-  </si>
-  <si>
-    <t>Max Mustermann</t>
-  </si>
-  <si>
-    <t>Susanne Muster</t>
-  </si>
-  <si>
-    <t>Felix Muster</t>
-  </si>
-  <si>
-    <t>Leon Mustermann</t>
-  </si>
-  <si>
-    <t>Renate Mustermann</t>
-  </si>
-  <si>
     <t>(insgesamt, d.h. Person selbst + zusätzliche Gäste)</t>
   </si>
   <si>
     <t>(gleicher Name wie bei Name)</t>
+  </si>
+  <si>
+    <t>Mustermann, Erika</t>
+  </si>
+  <si>
+    <t>Mustermann, Max</t>
+  </si>
+  <si>
+    <t>Muster, Susanne</t>
+  </si>
+  <si>
+    <t>Muster, Felix</t>
+  </si>
+  <si>
+    <t>Mustermann, Leon</t>
+  </si>
+  <si>
+    <t>Mustermann, Renate</t>
   </si>
 </sst>
 </file>
@@ -436,27 +436,24 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="B2">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>5</v>
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B3">
-        <v>5</v>
-      </c>
-      <c r="C3" t="s">
         <v>4</v>
-      </c>
-      <c r="D3" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -464,57 +461,60 @@
         <v>6</v>
       </c>
       <c r="B4">
-        <v>4</v>
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" t="s">
         <v>7</v>
-      </c>
-      <c r="B5">
-        <v>7</v>
-      </c>
-      <c r="C5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B6">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C6" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" t="s">
         <v>9</v>
-      </c>
-      <c r="D6" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B7">
         <v>2</v>
       </c>
       <c r="C7" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="C8" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="D8" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>